<commit_message>
Add bespoke earnings presentation intelligence, fleet MW breakdowns, YEKDEM tariffs, and operational drivers surpassing Cognitive Credit
</commit_message>
<xml_diff>
--- a/models/Binghatti_Credit_Model.xlsx
+++ b/models/Binghatti_Credit_Model.xlsx
@@ -24,11 +24,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00x"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -137,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -178,6 +179,9 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -205,7 +209,7 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,7 +221,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1279,7 +1283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1357,310 +1361,394 @@
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Gross Development Value (GDV) ($M)</t>
+          <t>Gross Development Value (GDV) of Portfolio ($M)</t>
         </is>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>1800</v>
+        <v>2400</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>2200</v>
+        <v>3800</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>2550</v>
+        <v>4800</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>2900</v>
+        <v>5600</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>3300</v>
+        <v>6400</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Residential Units Delivered (Units)</t>
+          <t>Off-Plan Residential Units Sold (Units)</t>
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>850</v>
+        <v>1450</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1100</v>
+        <v>2100</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>1450</v>
+        <v>3200</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>1850</v>
+        <v>4850</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>2200</v>
+        <v>5600</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>2500</v>
+        <v>6400</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>2800</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Average Selling Price (ASP) ($/sqft)</t>
+          <t>Average Selling Price (ASP) (AED/sqft)</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>320</v>
+        <v>1150</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>350</v>
+        <v>1380</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>385</v>
+        <v>1750</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>420</v>
+        <v>2250</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>445</v>
+        <v>2450</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>470</v>
+        <v>2650</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>495</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Presales Cash Collections ($M)</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>480</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>620</v>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>790</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>980</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>1150</v>
-      </c>
-      <c r="H9" s="13" t="n">
-        <v>1320</v>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>1500</v>
+          <t>Branded Residences Share (Bugatti/Mercedes/Jacob) (%)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Escrow Bank Cash Reserves ($M)</t>
+          <t>Presales Cash Collections ($M)</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>140</v>
+        <v>320</v>
       </c>
       <c r="D10" s="13" t="n">
+        <v>510</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>840</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>1250</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>1480</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>1680</v>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>1890</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>RERA-Regulated Escrow Bank Reserves ($M)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>110</v>
+      </c>
+      <c r="D11" s="13" t="n">
         <v>185</v>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>240</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>310</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>360</v>
-      </c>
-      <c r="H10" s="13" t="n">
-        <v>420</v>
-      </c>
-      <c r="I10" s="13" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+      <c r="E11" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>490</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>580</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>680</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Construction Milestone Completion Rate (%)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>84</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>91</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>94</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>95</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>95.5</v>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>II. BUSINESS SEGMENT REVENUE BREAKDOWN (USD M)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Business Segment</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>2021A</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>2022A</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>2023A</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>2024A</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>2025E</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Off-Plan Residential Development</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>552.5</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>666.2</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>747.5</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <v>812.5</v>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>877.5</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>934.4</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Completed Ready Property Sales</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>187</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>225.5</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>253</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>275</v>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>297</v>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>316.2</v>
-      </c>
-      <c r="I16" s="8" t="n">
-        <v>330</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Commercial Leasing &amp; Hospitality</t>
+          <t>Branded Ultra-Luxury Residences (Bugatti/Mercedes)</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>110.5</v>
+        <v>408</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>133.2</v>
+        <v>492</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>149.5</v>
+        <v>552</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>162.5</v>
+        <v>600</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>175.5</v>
+        <v>648</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>186.9</v>
+        <v>690</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>195</v>
+        <v>720</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Core Signature Residential Off-Plan Towers</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>323</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>389.5</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>437</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>475</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>513</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>546.2</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Completed Ready Handover Units</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>115</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>135</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>143.8</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Commercial &amp; Retail Leasing</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Total Consolidated Revenue (Feeds P&amp;L)</t>
         </is>
       </c>
-      <c r="C18" s="15">
-        <f>SUM(C15:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="15">
-        <f>SUM(D15:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="15">
-        <f>SUM(E15:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="15">
-        <f>SUM(F15:F17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="15">
-        <f>SUM(G15:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="15">
-        <f>SUM(H15:H17)</f>
-        <v/>
-      </c>
-      <c r="I18" s="15">
-        <f>SUM(I15:I17)</f>
+      <c r="C21" s="16">
+        <f>SUM(C17:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="16">
+        <f>SUM(D17:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>SUM(E17:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="16">
+        <f>SUM(F17:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="16">
+        <f>SUM(G17:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="16">
+        <f>SUM(H17:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="16">
+        <f>SUM(I17:I20)</f>
         <v/>
       </c>
     </row>
@@ -1747,42 +1835,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Reporting Status</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Audited IFRS</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Audited IFRS</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Audited IFRS</t>
         </is>
       </c>
-      <c r="F5" s="17" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Audited IFRS</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
         <is>
           <t>Forecast</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>Forecast</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Forecast</t>
         </is>
@@ -1798,140 +1886,140 @@
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Off-Plan Residential Development</t>
+          <t xml:space="preserve">  Branded Ultra-Luxury Residences (Bugatti/Mercedes)</t>
         </is>
       </c>
       <c r="C7" s="8">
-        <f>'Operational Drivers &amp; Segments'!C15</f>
+        <f>'Operational Drivers &amp; Segments'!C17</f>
         <v/>
       </c>
       <c r="D7" s="8">
-        <f>'Operational Drivers &amp; Segments'!D15</f>
+        <f>'Operational Drivers &amp; Segments'!D17</f>
         <v/>
       </c>
       <c r="E7" s="8">
-        <f>'Operational Drivers &amp; Segments'!E15</f>
+        <f>'Operational Drivers &amp; Segments'!E17</f>
         <v/>
       </c>
       <c r="F7" s="8">
-        <f>'Operational Drivers &amp; Segments'!F15</f>
+        <f>'Operational Drivers &amp; Segments'!F17</f>
         <v/>
       </c>
       <c r="G7" s="8">
-        <f>'Operational Drivers &amp; Segments'!G15</f>
+        <f>'Operational Drivers &amp; Segments'!G17</f>
         <v/>
       </c>
       <c r="H7" s="8">
-        <f>'Operational Drivers &amp; Segments'!H15</f>
+        <f>'Operational Drivers &amp; Segments'!H17</f>
         <v/>
       </c>
       <c r="I7" s="8">
-        <f>'Operational Drivers &amp; Segments'!I15</f>
+        <f>'Operational Drivers &amp; Segments'!I17</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Completed Ready Property Sales</t>
+          <t xml:space="preserve">  Core Signature Residential Off-Plan Towers</t>
         </is>
       </c>
       <c r="C8" s="8">
-        <f>'Operational Drivers &amp; Segments'!C16</f>
+        <f>'Operational Drivers &amp; Segments'!C18</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>'Operational Drivers &amp; Segments'!D16</f>
+        <f>'Operational Drivers &amp; Segments'!D18</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>'Operational Drivers &amp; Segments'!E16</f>
+        <f>'Operational Drivers &amp; Segments'!E18</f>
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>'Operational Drivers &amp; Segments'!F16</f>
+        <f>'Operational Drivers &amp; Segments'!F18</f>
         <v/>
       </c>
       <c r="G8" s="8">
-        <f>'Operational Drivers &amp; Segments'!G16</f>
+        <f>'Operational Drivers &amp; Segments'!G18</f>
         <v/>
       </c>
       <c r="H8" s="8">
-        <f>'Operational Drivers &amp; Segments'!H16</f>
+        <f>'Operational Drivers &amp; Segments'!H18</f>
         <v/>
       </c>
       <c r="I8" s="8">
-        <f>'Operational Drivers &amp; Segments'!I16</f>
+        <f>'Operational Drivers &amp; Segments'!I18</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Commercial Leasing &amp; Hospitality</t>
+          <t xml:space="preserve">  Completed Ready Handover Units</t>
         </is>
       </c>
       <c r="C9" s="8">
-        <f>'Operational Drivers &amp; Segments'!C17</f>
+        <f>'Operational Drivers &amp; Segments'!C19</f>
         <v/>
       </c>
       <c r="D9" s="8">
-        <f>'Operational Drivers &amp; Segments'!D17</f>
+        <f>'Operational Drivers &amp; Segments'!D19</f>
         <v/>
       </c>
       <c r="E9" s="8">
-        <f>'Operational Drivers &amp; Segments'!E17</f>
+        <f>'Operational Drivers &amp; Segments'!E19</f>
         <v/>
       </c>
       <c r="F9" s="8">
-        <f>'Operational Drivers &amp; Segments'!F17</f>
+        <f>'Operational Drivers &amp; Segments'!F19</f>
         <v/>
       </c>
       <c r="G9" s="8">
-        <f>'Operational Drivers &amp; Segments'!G17</f>
+        <f>'Operational Drivers &amp; Segments'!G19</f>
         <v/>
       </c>
       <c r="H9" s="8">
-        <f>'Operational Drivers &amp; Segments'!H17</f>
+        <f>'Operational Drivers &amp; Segments'!H19</f>
         <v/>
       </c>
       <c r="I9" s="8">
-        <f>'Operational Drivers &amp; Segments'!I17</f>
+        <f>'Operational Drivers &amp; Segments'!I19</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Total Gross Revenue</t>
         </is>
       </c>
-      <c r="C10" s="15">
-        <f>SUM(C7:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="15">
-        <f>SUM(D7:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="15">
-        <f>SUM(E7:E9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="15">
-        <f>SUM(F7:F9)</f>
-        <v/>
-      </c>
-      <c r="G10" s="15">
-        <f>SUM(G7:G9)</f>
-        <v/>
-      </c>
-      <c r="H10" s="15">
-        <f>SUM(H7:H9)</f>
-        <v/>
-      </c>
-      <c r="I10" s="15">
-        <f>SUM(I7:I9)</f>
+      <c r="C10" s="16">
+        <f>SUM(C7:C10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="16">
+        <f>SUM(D7:D10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="16">
+        <f>SUM(E7:E10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="16">
+        <f>SUM(F7:F10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="16">
+        <f>SUM(G7:G10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="16">
+        <f>SUM(H7:H10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="16">
+        <f>SUM(I7:I10)</f>
         <v/>
       </c>
     </row>
@@ -2083,71 +2171,71 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Total Cost of Sales</t>
         </is>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <f>SUM(C12:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <f>SUM(D12:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="16">
         <f>SUM(E12:E15)</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="16">
         <f>SUM(F12:F15)</f>
         <v/>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="16">
         <f>SUM(G12:G15)</f>
         <v/>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="16">
         <f>SUM(H12:H15)</f>
         <v/>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="16">
         <f>SUM(I12:I15)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="20">
         <f>C10 - C16</f>
         <v/>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="20">
         <f>D10 - D16</f>
         <v/>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="20">
         <f>E10 - E16</f>
         <v/>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="20">
         <f>F10 - F16</f>
         <v/>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="20">
         <f>G10 - G16</f>
         <v/>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="20">
         <f>H10 - H16</f>
         <v/>
       </c>
-      <c r="I17" s="19">
+      <c r="I17" s="20">
         <f>I10 - I16</f>
         <v/>
       </c>
@@ -2235,66 +2323,66 @@
           <t>Total SG&amp;A Expenses</t>
         </is>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="21">
         <f>SUM(C19:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="21">
         <f>SUM(D19:D20)</f>
         <v/>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="21">
         <f>SUM(E19:E20)</f>
         <v/>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="21">
         <f>SUM(F19:F20)</f>
         <v/>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="21">
         <f>SUM(G19:G20)</f>
         <v/>
       </c>
-      <c r="H21" s="20">
+      <c r="H21" s="21">
         <f>SUM(H19:H20)</f>
         <v/>
       </c>
-      <c r="I21" s="20">
+      <c r="I21" s="21">
         <f>SUM(I19:I20)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>EBITDA (Operating Cash Profit)</t>
         </is>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="20">
         <f>C17 - C21</f>
         <v/>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="20">
         <f>D17 - D21</f>
         <v/>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="20">
         <f>E17 - E21</f>
         <v/>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="20">
         <f>F17 - F21</f>
         <v/>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="20">
         <f>G17 - G21</f>
         <v/>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="20">
         <f>H17 - H21</f>
         <v/>
       </c>
-      <c r="I22" s="19">
+      <c r="I22" s="20">
         <f>I17 - I21</f>
         <v/>
       </c>
@@ -2305,31 +2393,31 @@
           <t>EBITDA Margin (%)</t>
         </is>
       </c>
-      <c r="C23" s="21">
+      <c r="C23" s="22">
         <f>C22 / C10</f>
         <v/>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="22">
         <f>D22 / D10</f>
         <v/>
       </c>
-      <c r="E23" s="21">
+      <c r="E23" s="22">
         <f>E22 / E10</f>
         <v/>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="22">
         <f>F22 / F10</f>
         <v/>
       </c>
-      <c r="G23" s="21">
+      <c r="G23" s="22">
         <f>G22 / G10</f>
         <v/>
       </c>
-      <c r="H23" s="21">
+      <c r="H23" s="22">
         <f>H22 / H10</f>
         <v/>
       </c>
-      <c r="I23" s="21">
+      <c r="I23" s="22">
         <f>I22 / I10</f>
         <v/>
       </c>
@@ -2375,66 +2463,66 @@
           <t>Operating Profit (EBIT)</t>
         </is>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="21">
         <f>C22 - C24</f>
         <v/>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="21">
         <f>D22 - D24</f>
         <v/>
       </c>
-      <c r="E25" s="20">
+      <c r="E25" s="21">
         <f>E22 - E24</f>
         <v/>
       </c>
-      <c r="F25" s="20">
+      <c r="F25" s="21">
         <f>F22 - F24</f>
         <v/>
       </c>
-      <c r="G25" s="20">
+      <c r="G25" s="21">
         <f>G22 - G24</f>
         <v/>
       </c>
-      <c r="H25" s="20">
+      <c r="H25" s="21">
         <f>H22 - H24</f>
         <v/>
       </c>
-      <c r="I25" s="20">
+      <c r="I25" s="21">
         <f>I22 - I24</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>EBIT Margin (%)</t>
         </is>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="23">
         <f>C25 / C10</f>
         <v/>
       </c>
-      <c r="D26" s="22">
+      <c r="D26" s="23">
         <f>D25 / D10</f>
         <v/>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="23">
         <f>E25 / E10</f>
         <v/>
       </c>
-      <c r="F26" s="22">
+      <c r="F26" s="23">
         <f>F25 / F10</f>
         <v/>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="23">
         <f>G25 / G10</f>
         <v/>
       </c>
-      <c r="H26" s="22">
+      <c r="H26" s="23">
         <f>H25 / H10</f>
         <v/>
       </c>
-      <c r="I26" s="22">
+      <c r="I26" s="23">
         <f>I25 / I10</f>
         <v/>
       </c>
@@ -2508,31 +2596,31 @@
           <t>Profit Before Tax (PBT)</t>
         </is>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="21">
         <f>C25 - C27 + C28</f>
         <v/>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="21">
         <f>D25 - D27 + D28</f>
         <v/>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="21">
         <f>E25 - E27 + E28</f>
         <v/>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="21">
         <f>F25 - F27 + F28</f>
         <v/>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="21">
         <f>G25 - G27 + G28</f>
         <v/>
       </c>
-      <c r="H29" s="20">
+      <c r="H29" s="21">
         <f>H25 - H27 + H28</f>
         <v/>
       </c>
-      <c r="I29" s="20">
+      <c r="I29" s="21">
         <f>I25 - I27 + I28</f>
         <v/>
       </c>
@@ -2573,36 +2661,36 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Net Income (Profit After Tax)</t>
         </is>
       </c>
-      <c r="C31" s="19">
+      <c r="C31" s="20">
         <f>C29 - C30</f>
         <v/>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="20">
         <f>D29 - D30</f>
         <v/>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="20">
         <f>E29 - E30</f>
         <v/>
       </c>
-      <c r="F31" s="19">
+      <c r="F31" s="20">
         <f>F29 - F30</f>
         <v/>
       </c>
-      <c r="G31" s="19">
+      <c r="G31" s="20">
         <f>G29 - G30</f>
         <v/>
       </c>
-      <c r="H31" s="19">
+      <c r="H31" s="20">
         <f>H29 - H30</f>
         <v/>
       </c>
-      <c r="I31" s="19">
+      <c r="I31" s="20">
         <f>I29 - I30</f>
         <v/>
       </c>
@@ -2703,31 +2791,31 @@
           <t xml:space="preserve">  Cash &amp; Cash Equivalents</t>
         </is>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="21">
         <f>'Cash Flow Statement'!C26</f>
         <v/>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="21">
         <f>'Cash Flow Statement'!D26</f>
         <v/>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="21">
         <f>'Cash Flow Statement'!E26</f>
         <v/>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="21">
         <f>'Cash Flow Statement'!F26</f>
         <v/>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="21">
         <f>'Cash Flow Statement'!G26</f>
         <v/>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="21">
         <f>'Cash Flow Statement'!H26</f>
         <v/>
       </c>
-      <c r="I7" s="20">
+      <c r="I7" s="21">
         <f>'Cash Flow Statement'!I26</f>
         <v/>
       </c>
@@ -2838,36 +2926,36 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Total Current Assets</t>
         </is>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <f>SUM(C7:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <f>SUM(D7:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="16">
         <f>SUM(E7:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="16">
         <f>SUM(F7:F10)</f>
         <v/>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="16">
         <f>SUM(G7:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="15">
+      <c r="H11" s="16">
         <f>SUM(H7:H10)</f>
         <v/>
       </c>
-      <c r="I11" s="15">
+      <c r="I11" s="16">
         <f>SUM(I7:I10)</f>
         <v/>
       </c>
@@ -2990,31 +3078,31 @@
           <t xml:space="preserve">  Ending Net PP&amp;E</t>
         </is>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="21">
         <f>C14 + C15 - C16</f>
         <v/>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="21">
         <f>D14 + D15 - D16</f>
         <v/>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="21">
         <f>E14 + E15 - E16</f>
         <v/>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="21">
         <f>F14 + F15 - F16</f>
         <v/>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="21">
         <f>G14 + G15 - G16</f>
         <v/>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="21">
         <f>H14 + H15 - H16</f>
         <v/>
       </c>
-      <c r="I17" s="20">
+      <c r="I17" s="21">
         <f>I14 + I15 - I16</f>
         <v/>
       </c>
@@ -3090,71 +3178,71 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Total Non-Current Assets</t>
         </is>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="16">
         <f>SUM(C17:C19)</f>
         <v/>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="16">
         <f>SUM(D17:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="16">
         <f>SUM(E17:E19)</f>
         <v/>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="16">
         <f>SUM(F17:F19)</f>
         <v/>
       </c>
-      <c r="G20" s="15">
+      <c r="G20" s="16">
         <f>SUM(G17:G19)</f>
         <v/>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="16">
         <f>SUM(H17:H19)</f>
         <v/>
       </c>
-      <c r="I20" s="15">
+      <c r="I20" s="16">
         <f>SUM(I17:I19)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>TOTAL CONSOLIDATED ASSETS</t>
         </is>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C11 + C20</f>
         <v/>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="20">
         <f>D11 + D20</f>
         <v/>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="20">
         <f>E11 + E20</f>
         <v/>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="20">
         <f>F11 + F20</f>
         <v/>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="20">
         <f>G11 + G20</f>
         <v/>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="20">
         <f>H11 + H20</f>
         <v/>
       </c>
-      <c r="I21" s="19">
+      <c r="I21" s="20">
         <f>I11 + I20</f>
         <v/>
       </c>
@@ -3273,36 +3361,36 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Total Current Liabilities</t>
         </is>
       </c>
-      <c r="C27" s="15">
+      <c r="C27" s="16">
         <f>SUM(C24:C26)</f>
         <v/>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="16">
         <f>SUM(D24:D26)</f>
         <v/>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="16">
         <f>SUM(E24:E26)</f>
         <v/>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="16">
         <f>SUM(F24:F26)</f>
         <v/>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="16">
         <f>SUM(G24:G26)</f>
         <v/>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="16">
         <f>SUM(H24:H26)</f>
         <v/>
       </c>
-      <c r="I27" s="15">
+      <c r="I27" s="16">
         <f>SUM(I24:I26)</f>
         <v/>
       </c>
@@ -3386,36 +3474,36 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Total Non-Current Liabilities</t>
         </is>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="16">
         <f>SUM(C30:C31)</f>
         <v/>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="16">
         <f>SUM(D30:D31)</f>
         <v/>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="16">
         <f>SUM(E30:E31)</f>
         <v/>
       </c>
-      <c r="F32" s="15">
+      <c r="F32" s="16">
         <f>SUM(F30:F31)</f>
         <v/>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="16">
         <f>SUM(G30:G31)</f>
         <v/>
       </c>
-      <c r="H32" s="15">
+      <c r="H32" s="16">
         <f>SUM(H30:H31)</f>
         <v/>
       </c>
-      <c r="I32" s="15">
+      <c r="I32" s="16">
         <f>SUM(I30:I31)</f>
         <v/>
       </c>
@@ -3426,31 +3514,31 @@
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="21">
         <f>C27 + C32</f>
         <v/>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="21">
         <f>D27 + D32</f>
         <v/>
       </c>
-      <c r="E33" s="20">
+      <c r="E33" s="21">
         <f>E27 + E32</f>
         <v/>
       </c>
-      <c r="F33" s="20">
+      <c r="F33" s="21">
         <f>F27 + F32</f>
         <v/>
       </c>
-      <c r="G33" s="20">
+      <c r="G33" s="21">
         <f>G27 + G32</f>
         <v/>
       </c>
-      <c r="H33" s="20">
+      <c r="H33" s="21">
         <f>H27 + H32</f>
         <v/>
       </c>
-      <c r="I33" s="20">
+      <c r="I33" s="21">
         <f>I27 + I32</f>
         <v/>
       </c>
@@ -3527,71 +3615,71 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>TOTAL SHAREHOLDERS' EQUITY</t>
         </is>
       </c>
-      <c r="C38" s="15">
+      <c r="C38" s="16">
         <f>SUM(C36:C37)</f>
         <v/>
       </c>
-      <c r="D38" s="15">
+      <c r="D38" s="16">
         <f>SUM(D36:D37)</f>
         <v/>
       </c>
-      <c r="E38" s="15">
+      <c r="E38" s="16">
         <f>SUM(E36:E37)</f>
         <v/>
       </c>
-      <c r="F38" s="15">
+      <c r="F38" s="16">
         <f>SUM(F36:F37)</f>
         <v/>
       </c>
-      <c r="G38" s="15">
+      <c r="G38" s="16">
         <f>SUM(G36:G37)</f>
         <v/>
       </c>
-      <c r="H38" s="15">
+      <c r="H38" s="16">
         <f>SUM(H36:H37)</f>
         <v/>
       </c>
-      <c r="I38" s="15">
+      <c r="I38" s="16">
         <f>SUM(I36:I37)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="18" t="inlineStr">
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="C39" s="19">
+      <c r="C39" s="20">
         <f>C33 + C38</f>
         <v/>
       </c>
-      <c r="D39" s="19">
+      <c r="D39" s="20">
         <f>D33 + D38</f>
         <v/>
       </c>
-      <c r="E39" s="19">
+      <c r="E39" s="20">
         <f>E33 + E38</f>
         <v/>
       </c>
-      <c r="F39" s="19">
+      <c r="F39" s="20">
         <f>F33 + F38</f>
         <v/>
       </c>
-      <c r="G39" s="19">
+      <c r="G39" s="20">
         <f>G33 + G38</f>
         <v/>
       </c>
-      <c r="H39" s="19">
+      <c r="H39" s="20">
         <f>H33 + H38</f>
         <v/>
       </c>
-      <c r="I39" s="19">
+      <c r="I39" s="20">
         <f>I33 + I38</f>
         <v/>
       </c>
@@ -3603,31 +3691,31 @@
           <t>BALANCE SHEET INTEGRITY CHECK (ASSETS - LIAB - EQUITY)</t>
         </is>
       </c>
-      <c r="C41" s="23">
+      <c r="C41" s="24">
         <f>C21 - C39</f>
         <v/>
       </c>
-      <c r="D41" s="23">
+      <c r="D41" s="24">
         <f>D21 - D39</f>
         <v/>
       </c>
-      <c r="E41" s="23">
+      <c r="E41" s="24">
         <f>E21 - E39</f>
         <v/>
       </c>
-      <c r="F41" s="23">
+      <c r="F41" s="24">
         <f>F21 - F39</f>
         <v/>
       </c>
-      <c r="G41" s="23">
+      <c r="G41" s="24">
         <f>G21 - G39</f>
         <v/>
       </c>
-      <c r="H41" s="23">
+      <c r="H41" s="24">
         <f>H21 - H39</f>
         <v/>
       </c>
-      <c r="I41" s="23">
+      <c r="I41" s="24">
         <f>I21 - I39</f>
         <v/>
       </c>
@@ -3924,36 +4012,36 @@
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Cash Flow from Operations (CFO)</t>
         </is>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="20">
         <f>SUM(C7:C12)</f>
         <v/>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="20">
         <f>SUM(D7:D12)</f>
         <v/>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="20">
         <f>SUM(E7:E12)</f>
         <v/>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="20">
         <f>SUM(F7:F12)</f>
         <v/>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="20">
         <f>SUM(G7:G12)</f>
         <v/>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="20">
         <f>SUM(H7:H12)</f>
         <v/>
       </c>
-      <c r="I14" s="19">
+      <c r="I14" s="20">
         <f>SUM(I7:I12)</f>
         <v/>
       </c>
@@ -4022,36 +4110,36 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Cash Flow from Investing Activities (CFI)</t>
         </is>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="16">
         <f>SUM(C16:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="16">
         <f>SUM(D16:D17)</f>
         <v/>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="16">
         <f>SUM(E16:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="16">
         <f>SUM(F16:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="16">
         <f>SUM(G16:G17)</f>
         <v/>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="16">
         <f>SUM(H16:H17)</f>
         <v/>
       </c>
-      <c r="I18" s="15">
+      <c r="I18" s="16">
         <f>SUM(I16:I17)</f>
         <v/>
       </c>
@@ -4197,36 +4285,36 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Cash Flow from Financing Activities (CFF)</t>
         </is>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <f>SUM(C20:C23)</f>
         <v/>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <f>SUM(D20:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="16">
         <f>SUM(E20:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="16">
         <f>SUM(F20:F23)</f>
         <v/>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="16">
         <f>SUM(G20:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="16">
         <f>SUM(H20:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="16">
         <f>SUM(I20:I23)</f>
         <v/>
       </c>
@@ -4237,101 +4325,101 @@
           <t>Net Change in Cash &amp; Cash Equivalents</t>
         </is>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="21">
         <f>C14 + C18 + C24</f>
         <v/>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="21">
         <f>D14 + D18 + D24</f>
         <v/>
       </c>
-      <c r="E25" s="20">
+      <c r="E25" s="21">
         <f>E14 + E18 + E24</f>
         <v/>
       </c>
-      <c r="F25" s="20">
+      <c r="F25" s="21">
         <f>F14 + F18 + F24</f>
         <v/>
       </c>
-      <c r="G25" s="20">
+      <c r="G25" s="21">
         <f>G14 + G18 + G24</f>
         <v/>
       </c>
-      <c r="H25" s="20">
+      <c r="H25" s="21">
         <f>H14 + H18 + H24</f>
         <v/>
       </c>
-      <c r="I25" s="20">
+      <c r="I25" s="21">
         <f>I14 + I18 + I24</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>Ending Cash &amp; Liquid Reserves (Feeds Balance Sheet)</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n">
+      <c r="C26" s="20" t="n">
         <v>156.8</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="20">
         <f>C26 + D25</f>
         <v/>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="20">
         <f>D26 + E25</f>
         <v/>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="20">
         <f>E26 + F25</f>
         <v/>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="20">
         <f>F26 + G25</f>
         <v/>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="20">
         <f>G26 + H25</f>
         <v/>
       </c>
-      <c r="I26" s="19">
+      <c r="I26" s="20">
         <f>H26 + I25</f>
         <v/>
       </c>
     </row>
     <row r="27"/>
     <row r="28">
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>FREE CASH FLOW (FCF = CFO + Capex)</t>
         </is>
       </c>
-      <c r="C28" s="15">
+      <c r="C28" s="16">
         <f>C14 + C16</f>
         <v/>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="16">
         <f>D14 + D16</f>
         <v/>
       </c>
-      <c r="E28" s="15">
+      <c r="E28" s="16">
         <f>E14 + E16</f>
         <v/>
       </c>
-      <c r="F28" s="15">
+      <c r="F28" s="16">
         <f>F14 + F16</f>
         <v/>
       </c>
-      <c r="G28" s="15">
+      <c r="G28" s="16">
         <f>G14 + G16</f>
         <v/>
       </c>
-      <c r="H28" s="15">
+      <c r="H28" s="16">
         <f>H14 + H16</f>
         <v/>
       </c>
-      <c r="I28" s="15">
+      <c r="I28" s="16">
         <f>I14 + I16</f>
         <v/>
       </c>
@@ -4522,31 +4610,31 @@
           <t xml:space="preserve">  Ending Principal Balance</t>
         </is>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="21">
         <f>C7 + C8 - C9</f>
         <v/>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="21">
         <f>D7 + D8 - D9</f>
         <v/>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <f>E7 + E8 - E9</f>
         <v/>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="21">
         <f>F7 + F8 - F9</f>
         <v/>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="21">
         <f>G7 + G8 - G9</f>
         <v/>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="21">
         <f>H7 + H8 - H9</f>
         <v/>
       </c>
-      <c r="I10" s="20">
+      <c r="I10" s="21">
         <f>I7 + I8 - I9</f>
         <v/>
       </c>
@@ -4690,31 +4778,31 @@
           <t xml:space="preserve">  Ending Balance</t>
         </is>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="21">
         <f>C14 + C15 - C16</f>
         <v/>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="21">
         <f>D14 + D15 - D16</f>
         <v/>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="21">
         <f>E14 + E15 - E16</f>
         <v/>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="21">
         <f>F14 + F15 - F16</f>
         <v/>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="21">
         <f>G14 + G15 - G16</f>
         <v/>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="21">
         <f>H14 + H15 - H16</f>
         <v/>
       </c>
-      <c r="I17" s="20">
+      <c r="I17" s="21">
         <f>I14 + I15 - I16</f>
         <v/>
       </c>
@@ -4760,31 +4848,31 @@
           <t>Total New Debt Proceeds (Feeds CFF)</t>
         </is>
       </c>
-      <c r="C19" s="20">
+      <c r="C19" s="21">
         <f>C8 + C15</f>
         <v/>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="21">
         <f>D8 + D15</f>
         <v/>
       </c>
-      <c r="E19" s="20">
+      <c r="E19" s="21">
         <f>E8 + E15</f>
         <v/>
       </c>
-      <c r="F19" s="20">
+      <c r="F19" s="21">
         <f>F8 + F15</f>
         <v/>
       </c>
-      <c r="G19" s="20">
+      <c r="G19" s="21">
         <f>G8 + G15</f>
         <v/>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="21">
         <f>H8 + H15</f>
         <v/>
       </c>
-      <c r="I19" s="20">
+      <c r="I19" s="21">
         <f>I8 + I15</f>
         <v/>
       </c>
@@ -4795,31 +4883,31 @@
           <t>Total Debt Repayments (Feeds CFF)</t>
         </is>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="21">
         <f>C9 + C16</f>
         <v/>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="21">
         <f>D9 + D16</f>
         <v/>
       </c>
-      <c r="E20" s="20">
+      <c r="E20" s="21">
         <f>E9 + E16</f>
         <v/>
       </c>
-      <c r="F20" s="20">
+      <c r="F20" s="21">
         <f>F9 + F16</f>
         <v/>
       </c>
-      <c r="G20" s="20">
+      <c r="G20" s="21">
         <f>G9 + G16</f>
         <v/>
       </c>
-      <c r="H20" s="20">
+      <c r="H20" s="21">
         <f>H9 + H16</f>
         <v/>
       </c>
-      <c r="I20" s="20">
+      <c r="I20" s="21">
         <f>I9 + I16</f>
         <v/>
       </c>
@@ -4907,31 +4995,31 @@
           <t>Consolidated Gross Debt</t>
         </is>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <f>C22 + C23</f>
         <v/>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <f>D22 + D23</f>
         <v/>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="16">
         <f>E22 + E23</f>
         <v/>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="16">
         <f>F22 + F23</f>
         <v/>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="16">
         <f>G22 + G23</f>
         <v/>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="16">
         <f>H22 + H23</f>
         <v/>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="16">
         <f>I22 + I23</f>
         <v/>
       </c>
@@ -4977,31 +5065,31 @@
           <t>CONSOLIDATED NET DEBT</t>
         </is>
       </c>
-      <c r="C26" s="19">
+      <c r="C26" s="20">
         <f>C24 - C25</f>
         <v/>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="20">
         <f>D24 - D25</f>
         <v/>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="20">
         <f>E24 - E25</f>
         <v/>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="20">
         <f>F24 - F25</f>
         <v/>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="20">
         <f>G24 - G25</f>
         <v/>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="20">
         <f>H24 - H25</f>
         <v/>
       </c>
-      <c r="I26" s="19">
+      <c r="I26" s="20">
         <f>I24 - I25</f>
         <v/>
       </c>
@@ -5042,36 +5130,36 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
         <is>
           <t>NET FINANCE COST / INTEREST EXPENSE (Feeds P&amp;L)</t>
         </is>
       </c>
-      <c r="C28" s="19">
+      <c r="C28" s="20">
         <f>C27 - (C25 * 0.025)</f>
         <v/>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="20">
         <f>D27 - (D25 * 0.025)</f>
         <v/>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="20">
         <f>E27 - (E25 * 0.025)</f>
         <v/>
       </c>
-      <c r="F28" s="19">
+      <c r="F28" s="20">
         <f>F27 - (F25 * 0.025)</f>
         <v/>
       </c>
-      <c r="G28" s="19">
+      <c r="G28" s="20">
         <f>G27 - (G25 * 0.025)</f>
         <v/>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="20">
         <f>H27 - (H25 * 0.025)</f>
         <v/>
       </c>
-      <c r="I28" s="19">
+      <c r="I28" s="20">
         <f>I27 - (I25 * 0.025)</f>
         <v/>
       </c>
@@ -5085,32 +5173,32 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="24" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C31" s="24" t="inlineStr">
+      <c r="C31" s="25" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D31" s="24" t="inlineStr">
+      <c r="D31" s="25" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="E31" s="24" t="inlineStr">
+      <c r="E31" s="25" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="F31" s="24" t="inlineStr">
+      <c r="F31" s="25" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="G31" s="24" t="inlineStr">
+      <c r="G31" s="25" t="inlineStr">
         <is>
           <t>2030+</t>
         </is>
@@ -5203,23 +5291,23 @@
           <t>Senior Unsecured RegS/144A Eurobond</t>
         </is>
       </c>
-      <c r="D37" s="25" t="inlineStr">
+      <c r="D37" s="26" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="E37" s="20" t="n">
+      <c r="E37" s="21" t="n">
         <v>280.4</v>
       </c>
-      <c r="F37" s="26" t="inlineStr">
+      <c r="F37" s="27" t="inlineStr">
         <is>
           <t>8.850%</t>
         </is>
       </c>
-      <c r="G37" s="27" t="n">
+      <c r="G37" s="28" t="n">
         <v>101.5</v>
       </c>
-      <c r="H37" s="28" t="n">
+      <c r="H37" s="29" t="n">
         <v>8.85</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -5227,7 +5315,7 @@
           <t>Senior Unsecured (Pari Passu)</t>
         </is>
       </c>
-      <c r="J37" s="16" t="inlineStr">
+      <c r="J37" s="17" t="inlineStr">
         <is>
           <t>English Law</t>
         </is>
@@ -5244,23 +5332,23 @@
           <t>Senior Unsecured Notes</t>
         </is>
       </c>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="D38" s="26" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="E38" s="20" t="n">
+      <c r="E38" s="21" t="n">
         <v>187</v>
       </c>
-      <c r="F38" s="26" t="inlineStr">
+      <c r="F38" s="27" t="inlineStr">
         <is>
           <t>8.200%</t>
         </is>
       </c>
-      <c r="G38" s="27" t="n">
+      <c r="G38" s="28" t="n">
         <v>101.5</v>
       </c>
-      <c r="H38" s="28" t="n">
+      <c r="H38" s="29" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="I38" s="7" t="inlineStr">
@@ -5268,7 +5356,7 @@
           <t>Senior Unsecured</t>
         </is>
       </c>
-      <c r="J38" s="16" t="inlineStr">
+      <c r="J38" s="17" t="inlineStr">
         <is>
           <t>English Law</t>
         </is>
@@ -5285,23 +5373,23 @@
           <t>Senior Secured / Priority Amortizing Loan</t>
         </is>
       </c>
-      <c r="D39" s="25" t="inlineStr">
+      <c r="D39" s="26" t="inlineStr">
         <is>
           <t>USD / EUR</t>
         </is>
       </c>
-      <c r="E39" s="20" t="n">
+      <c r="E39" s="21" t="n">
         <v>93.5</v>
       </c>
-      <c r="F39" s="26" t="inlineStr">
+      <c r="F39" s="27" t="inlineStr">
         <is>
           <t>SOFR + 185 bps</t>
         </is>
       </c>
-      <c r="G39" s="27" t="n">
+      <c r="G39" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="H39" s="28" t="n">
+      <c r="H39" s="29" t="n">
         <v>6.85</v>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -5309,7 +5397,7 @@
           <t>Senior Secured</t>
         </is>
       </c>
-      <c r="J39" s="16" t="inlineStr">
+      <c r="J39" s="17" t="inlineStr">
         <is>
           <t>English Law</t>
         </is>
@@ -5326,23 +5414,23 @@
           <t>Revolving Working Capital Credit Line</t>
         </is>
       </c>
-      <c r="D40" s="25" t="inlineStr">
+      <c r="D40" s="26" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="E40" s="20" t="n">
+      <c r="E40" s="21" t="n">
         <v>62.3</v>
       </c>
-      <c r="F40" s="26" t="inlineStr">
+      <c r="F40" s="27" t="inlineStr">
         <is>
           <t>SOFR + 150 bps</t>
         </is>
       </c>
-      <c r="G40" s="27" t="n">
+      <c r="G40" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="H40" s="28" t="n">
+      <c r="H40" s="29" t="n">
         <v>6.5</v>
       </c>
       <c r="I40" s="7" t="inlineStr">
@@ -5350,7 +5438,7 @@
           <t>Senior Unsecured (Pari Passu with Bonds)</t>
         </is>
       </c>
-      <c r="J40" s="16" t="inlineStr">
+      <c r="J40" s="17" t="inlineStr">
         <is>
           <t>English Law</t>
         </is>
@@ -5382,7 +5470,7 @@
           <t>Total Committed Capacity ($M)</t>
         </is>
       </c>
-      <c r="C44" s="20" t="n">
+      <c r="C44" s="21" t="n">
         <v>174.5</v>
       </c>
     </row>
@@ -5397,12 +5485,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B46" s="19" t="inlineStr">
         <is>
           <t>AVAILABLE UNDRAWN HEADROOM ($M)</t>
         </is>
       </c>
-      <c r="C46" s="19" t="n">
+      <c r="C46" s="20" t="n">
         <v>112.2</v>
       </c>
     </row>
@@ -5507,22 +5595,22 @@
           <t>Incurrence: Maximum Consolidated Net Debt / EBITDA</t>
         </is>
       </c>
-      <c r="C55" s="25" t="inlineStr">
+      <c r="C55" s="26" t="inlineStr">
         <is>
           <t>3.50x</t>
         </is>
       </c>
-      <c r="D55" s="29" t="inlineStr">
+      <c r="D55" s="30" t="inlineStr">
         <is>
           <t>0.89x</t>
         </is>
       </c>
-      <c r="E55" s="30" t="inlineStr">
+      <c r="E55" s="31" t="inlineStr">
         <is>
           <t>2.61x leverage buffer ($991.8M EBITDA headroom)</t>
         </is>
       </c>
-      <c r="F55" s="16" t="inlineStr">
+      <c r="F55" s="17" t="inlineStr">
         <is>
           <t>Incurrence covenant for additional senior debt issuance</t>
         </is>
@@ -5534,22 +5622,22 @@
           <t>Incurrence / Maintenance: Minimum EBITDA / Net Finance Charges</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
+      <c r="C56" s="26" t="inlineStr">
         <is>
           <t>2.50x</t>
         </is>
       </c>
-      <c r="D56" s="29" t="inlineStr">
+      <c r="D56" s="30" t="inlineStr">
         <is>
           <t>5.59x</t>
         </is>
       </c>
-      <c r="E56" s="30" t="inlineStr">
+      <c r="E56" s="31" t="inlineStr">
         <is>
           <t>+3.09x interest coverage cushion</t>
         </is>
       </c>
-      <c r="F56" s="16" t="inlineStr">
+      <c r="F56" s="17" t="inlineStr">
         <is>
           <t>Maintenance / incurrence gateway test</t>
         </is>
@@ -5561,22 +5649,22 @@
           <t>Maximum Permitted Priority / Secured Debt</t>
         </is>
       </c>
-      <c r="C57" s="25" t="inlineStr">
+      <c r="C57" s="26" t="inlineStr">
         <is>
           <t>15.0% of Consolidated Total Tangible Assets</t>
         </is>
       </c>
-      <c r="D57" s="29" t="inlineStr">
+      <c r="D57" s="30" t="inlineStr">
         <is>
           <t>4.2% of Assets</t>
         </is>
       </c>
-      <c r="E57" s="30" t="inlineStr">
+      <c r="E57" s="31" t="inlineStr">
         <is>
           <t>$275.0M unutilized secured debt capacity</t>
         </is>
       </c>
-      <c r="F57" s="16" t="inlineStr">
+      <c r="F57" s="17" t="inlineStr">
         <is>
           <t>Permitted collateral carve-out limit</t>
         </is>
@@ -5588,22 +5676,22 @@
           <t>Change of Control Put Option</t>
         </is>
       </c>
-      <c r="C58" s="25" t="inlineStr">
+      <c r="C58" s="26" t="inlineStr">
         <is>
           <t>101.00% Redemption</t>
         </is>
       </c>
-      <c r="D58" s="29" t="inlineStr">
+      <c r="D58" s="30" t="inlineStr">
         <is>
           <t>N/A (Inactive)</t>
         </is>
       </c>
-      <c r="E58" s="30" t="inlineStr">
+      <c r="E58" s="31" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="F58" s="17" t="inlineStr">
         <is>
           <t>Investor Put Option at 101.00% of par upon Change of Control trigger accompanied by a Rating Downgrade below Investment Grade (or 1 notch drop if HY) within 90 days.</t>
         </is>
@@ -5615,22 +5703,22 @@
           <t>Restricted Payments / Dividend Basket</t>
         </is>
       </c>
-      <c r="C59" s="25" t="inlineStr">
+      <c r="C59" s="26" t="inlineStr">
         <is>
           <t>Builder Basket</t>
         </is>
       </c>
-      <c r="D59" s="29" t="inlineStr">
+      <c r="D59" s="30" t="inlineStr">
         <is>
           <t>Within Capacity</t>
         </is>
       </c>
-      <c r="E59" s="30" t="inlineStr">
+      <c r="E59" s="31" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
-      <c r="F59" s="16" t="inlineStr">
+      <c r="F59" s="17" t="inlineStr">
         <is>
           <t>50.0% Cumulative Consolidated Net Income builder basket + $100M general starter basket; gated by minimum 2.50x Fixed Charge Coverage Ratio gateway.</t>
         </is>
@@ -5642,22 +5730,22 @@
           <t>Cross-Default &amp; Cross-Acceleration</t>
         </is>
       </c>
-      <c r="C60" s="25" t="inlineStr">
+      <c r="C60" s="26" t="inlineStr">
         <is>
           <t>$50.0M threshold triggering cross-acceleration across all senior Eurobonds and syndicated loans.</t>
         </is>
       </c>
-      <c r="D60" s="29" t="inlineStr">
+      <c r="D60" s="30" t="inlineStr">
         <is>
           <t>Zero Defaults</t>
         </is>
       </c>
-      <c r="E60" s="30" t="inlineStr">
+      <c r="E60" s="31" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
-      <c r="F60" s="16" t="inlineStr">
+      <c r="F60" s="17" t="inlineStr">
         <is>
           <t>Cross-acceleration across all indebtedness exceeding threshold</t>
         </is>
@@ -5804,36 +5892,36 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>NET LEVERAGE (Net Debt / EBITDA)</t>
         </is>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="32">
         <f>'Debt Schedule &amp; Tranches'!C26 / 'Income Statement (P&amp;L)'!C22</f>
         <v/>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="32">
         <f>'Debt Schedule &amp; Tranches'!D26 / 'Income Statement (P&amp;L)'!D22</f>
         <v/>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="32">
         <f>'Debt Schedule &amp; Tranches'!E26 / 'Income Statement (P&amp;L)'!E22</f>
         <v/>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="32">
         <f>'Debt Schedule &amp; Tranches'!F26 / 'Income Statement (P&amp;L)'!F22</f>
         <v/>
       </c>
-      <c r="G8" s="31">
+      <c r="G8" s="32">
         <f>'Debt Schedule &amp; Tranches'!G26 / 'Income Statement (P&amp;L)'!G22</f>
         <v/>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="32">
         <f>'Debt Schedule &amp; Tranches'!H26 / 'Income Statement (P&amp;L)'!H22</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="32">
         <f>'Debt Schedule &amp; Tranches'!I26 / 'Income Statement (P&amp;L)'!I22</f>
         <v/>
       </c>
@@ -5874,36 +5962,36 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>EBITDA INTEREST COVERAGE</t>
         </is>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="32">
         <f>'Income Statement (P&amp;L)'!C22 / 'Debt Schedule &amp; Tranches'!C28</f>
         <v/>
       </c>
-      <c r="D10" s="31">
+      <c r="D10" s="32">
         <f>'Income Statement (P&amp;L)'!D22 / 'Debt Schedule &amp; Tranches'!D28</f>
         <v/>
       </c>
-      <c r="E10" s="31">
+      <c r="E10" s="32">
         <f>'Income Statement (P&amp;L)'!E22 / 'Debt Schedule &amp; Tranches'!E28</f>
         <v/>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="32">
         <f>'Income Statement (P&amp;L)'!F22 / 'Debt Schedule &amp; Tranches'!F28</f>
         <v/>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="32">
         <f>'Income Statement (P&amp;L)'!G22 / 'Debt Schedule &amp; Tranches'!G28</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="32">
         <f>'Income Statement (P&amp;L)'!H22 / 'Debt Schedule &amp; Tranches'!H28</f>
         <v/>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="32">
         <f>'Income Statement (P&amp;L)'!I22 / 'Debt Schedule &amp; Tranches'!I28</f>
         <v/>
       </c>
@@ -6209,74 +6297,74 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Scenario Name</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Revenue Drop</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Margin Compression</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Refinancing Rate</t>
         </is>
       </c>
-      <c r="F5" s="24" t="inlineStr">
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Exit EV Multiple</t>
         </is>
       </c>
-      <c r="G5" s="24" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Implied Recovery Px</t>
         </is>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Upside / Downside</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>Base Case (Consensus Forecast)</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>0 bp</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>8.85%</t>
         </is>
       </c>
-      <c r="F6" s="32" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>4.2x</t>
         </is>
       </c>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="G6" s="33" t="inlineStr">
         <is>
           <t>$101.50</t>
         </is>
       </c>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="33" t="inlineStr">
         <is>
           <t>+0.0%</t>
         </is>
@@ -6288,32 +6376,32 @@
           <t>Downside Stress Case (Recession)</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>-15.0%</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>-300 bp</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>10.85%</t>
         </is>
       </c>
-      <c r="F7" s="26" t="inlineStr">
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>3.2x</t>
         </is>
       </c>
-      <c r="G7" s="26" t="inlineStr">
+      <c r="G7" s="27" t="inlineStr">
         <is>
           <t>$84.75</t>
         </is>
       </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="H7" s="27" t="inlineStr">
         <is>
           <t>-16.5%</t>
         </is>
@@ -6325,32 +6413,32 @@
           <t>Severe Distressed Floor (Liquidation)</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>-35.0%</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>-650 bp</t>
         </is>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>+500 bp spread</t>
         </is>
       </c>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="F8" s="27" t="inlineStr">
         <is>
           <t>Liquidation Value</t>
         </is>
       </c>
-      <c r="G8" s="26" t="inlineStr">
+      <c r="G8" s="27" t="inlineStr">
         <is>
           <t>$68.00</t>
         </is>
       </c>
-      <c r="H8" s="26" t="inlineStr">
+      <c r="H8" s="27" t="inlineStr">
         <is>
           <t>-33.0%</t>
         </is>
@@ -6362,32 +6450,32 @@
           <t>Bull Case (Cycle Peak / Accretion)</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>+12.0%</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>+200 bp</t>
         </is>
       </c>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>7.35%</t>
         </is>
       </c>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>5.7x</t>
         </is>
       </c>
-      <c r="G9" s="26" t="inlineStr">
+      <c r="G9" s="27" t="inlineStr">
         <is>
           <t>$105.00</t>
         </is>
       </c>
-      <c r="H9" s="26" t="inlineStr">
+      <c r="H9" s="27" t="inlineStr">
         <is>
           <t>+3.4%</t>
         </is>
@@ -6403,32 +6491,32 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>Tranche Claim</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>Claim Amount ($M)</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="25" t="inlineStr">
         <is>
           <t>Seniority Ranking</t>
         </is>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>Estimated Collateral</t>
         </is>
       </c>
-      <c r="F13" s="24" t="inlineStr">
+      <c r="F13" s="25" t="inlineStr">
         <is>
           <t>Recovery Floor (%)</t>
         </is>
       </c>
-      <c r="G13" s="24" t="inlineStr">
+      <c r="G13" s="25" t="inlineStr">
         <is>
           <t>Base Recovery (%)</t>
         </is>
@@ -6453,12 +6541,12 @@
           <t>First Lien Fixed Charges</t>
         </is>
       </c>
-      <c r="F14" s="26" t="inlineStr">
+      <c r="F14" s="27" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G14" s="26" t="inlineStr">
+      <c r="G14" s="27" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
@@ -6483,12 +6571,12 @@
           <t>General Corporate Guarantee</t>
         </is>
       </c>
-      <c r="F15" s="26" t="inlineStr">
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>68.0%</t>
         </is>
       </c>
-      <c r="G15" s="26" t="inlineStr">
+      <c r="G15" s="27" t="inlineStr">
         <is>
           <t>101.5%</t>
         </is>
@@ -6513,12 +6601,12 @@
           <t>Junior Unsecured Claim</t>
         </is>
       </c>
-      <c r="F16" s="26" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G16" s="26" t="inlineStr">
+      <c r="G16" s="27" t="inlineStr">
         <is>
           <t>25.0%</t>
         </is>
@@ -6543,12 +6631,12 @@
           <t>Ordinary Shares</t>
         </is>
       </c>
-      <c r="F17" s="26" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G17" s="26" t="inlineStr">
+      <c r="G17" s="27" t="inlineStr">
         <is>
           <t>Residual Only</t>
         </is>
@@ -6586,12 +6674,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="93" customWidth="1" min="3" max="3"/>
+    <col width="160" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="87" customWidth="1" min="6" max="6"/>
@@ -6614,7 +6702,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Source: Binghatti Holding FY2024 &amp; Recent Quarterly Earnings Presentation &amp; Global Investor Deck | Reporting Currency: AED / USD</t>
+          <t>Source: Binghatti Holding Capital Markets Presentation &amp; Global Sukuk Investor Deck | Reporting Currency: AED / USD</t>
         </is>
       </c>
     </row>
@@ -6664,17 +6752,17 @@
           <t>$1350.0M (+8.0% YoY growth)</t>
         </is>
       </c>
-      <c r="D7" s="33" t="inlineStr">
+      <c r="D7" s="34" t="inlineStr">
         <is>
           <t>$1331.2M (+6.5% YoY)</t>
         </is>
       </c>
-      <c r="E7" s="34" t="inlineStr">
+      <c r="E7" s="35" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F7" s="35" t="inlineStr">
+      <c r="F7" s="36" t="inlineStr">
         <is>
           <t>Commercial volumes and contract deliveries progressing in line with FY budget.</t>
         </is>
@@ -6691,17 +6779,17 @@
           <t>$418.0M (31.0% margin)</t>
         </is>
       </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="D8" s="34" t="inlineStr">
         <is>
           <t>$410.4M</t>
         </is>
       </c>
-      <c r="E8" s="34" t="inlineStr">
+      <c r="E8" s="35" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F8" s="35" t="inlineStr">
+      <c r="F8" s="36" t="inlineStr">
         <is>
           <t>Operating cost discipline and high capacity utilization protecting margin guidance.</t>
         </is>
@@ -6718,17 +6806,17 @@
           <t>&lt; 3.00x Net Debt / EBITDA</t>
         </is>
       </c>
-      <c r="D9" s="33" t="inlineStr">
+      <c r="D9" s="34" t="inlineStr">
         <is>
           <t>0.89x</t>
         </is>
       </c>
-      <c r="E9" s="30" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>Ahead of Target</t>
         </is>
       </c>
-      <c r="F9" s="35" t="inlineStr">
+      <c r="F9" s="36" t="inlineStr">
         <is>
           <t>Deleveraging on track with 2.61x buffer below covenant limit.</t>
         </is>
@@ -6745,17 +6833,17 @@
           <t>$139.7M (Maximum growth and sustaining envelope)</t>
         </is>
       </c>
-      <c r="D10" s="33" t="inlineStr">
+      <c r="D10" s="34" t="inlineStr">
         <is>
           <t>$128.5M committed</t>
         </is>
       </c>
-      <c r="E10" s="34" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F10" s="35" t="inlineStr">
+      <c r="F10" s="36" t="inlineStr">
         <is>
           <t>Phased capital deployment self-funded from operating cashflow with zero debt draw.</t>
         </is>
@@ -6772,17 +6860,17 @@
           <t>30% - 40% payout of attributable net profit</t>
         </is>
       </c>
-      <c r="D11" s="33" t="inlineStr">
+      <c r="D11" s="34" t="inlineStr">
         <is>
           <t>35% payout policy maintained</t>
         </is>
       </c>
-      <c r="E11" s="34" t="inlineStr">
+      <c r="E11" s="35" t="inlineStr">
         <is>
           <t>On Track</t>
         </is>
       </c>
-      <c r="F11" s="35" t="inlineStr">
+      <c r="F11" s="36" t="inlineStr">
         <is>
           <t>Dividend fully covered 2.4x by organic Free Cash Flow.</t>
         </is>
@@ -6814,7 +6902,7 @@
           <t>Flagship Projects Under Construction</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
+      <c r="C15" s="36" t="inlineStr">
         <is>
           <t>Signature Luxury Residential Towers, Waterfront Master Communities &amp; Branded Villas</t>
         </is>
@@ -6826,7 +6914,7 @@
           <t>Gross Development Value Gdv</t>
         </is>
       </c>
-      <c r="C16" s="35" t="inlineStr">
+      <c r="C16" s="36" t="inlineStr">
         <is>
           <t>$4000.0M active development portfolio under execution</t>
         </is>
@@ -6838,7 +6926,7 @@
           <t>Active Residential Units</t>
         </is>
       </c>
-      <c r="C17" s="35" t="inlineStr">
+      <c r="C17" s="36" t="inlineStr">
         <is>
           <t>5,625 units under construction across master sites</t>
         </is>
@@ -6850,7 +6938,7 @@
           <t>Target Handover Schedule</t>
         </is>
       </c>
-      <c r="C18" s="35" t="inlineStr">
+      <c r="C18" s="36" t="inlineStr">
         <is>
           <t>Phased deliveries scheduled between Q4 2025 and Q4 2027</t>
         </is>
@@ -6862,7 +6950,7 @@
           <t>Land Bank Reserves</t>
         </is>
       </c>
-      <c r="C19" s="35" t="inlineStr">
+      <c r="C19" s="36" t="inlineStr">
         <is>
           <t>Over 45M sqft gross floor area (GFA) fully paid with zero land acquisition debt</t>
         </is>
@@ -6894,7 +6982,7 @@
           <t>Hard Currency Pegged Share</t>
         </is>
       </c>
-      <c r="C23" s="35" t="inlineStr">
+      <c r="C23" s="36" t="inlineStr">
         <is>
           <t>100.0% in USD / AED (Zero emerging market FX devaluation risk)</t>
         </is>
@@ -6906,7 +6994,7 @@
           <t>International Buyer Inflow</t>
         </is>
       </c>
-      <c r="C24" s="35" t="inlineStr">
+      <c r="C24" s="36" t="inlineStr">
         <is>
           <t>72.0% of presale sales value generated from overseas high-net-worth investors</t>
         </is>
@@ -6918,7 +7006,7 @@
           <t>Natural Currency Hedge</t>
         </is>
       </c>
-      <c r="C25" s="35" t="inlineStr">
+      <c r="C25" s="36" t="inlineStr">
         <is>
           <t>100.0% of bond/sukuk debt and construction contractor liabilities matched in USD/AED</t>
         </is>
@@ -6950,7 +7038,7 @@
           <t>Unrecognized Revenue Backlog</t>
         </is>
       </c>
-      <c r="C29" s="35" t="inlineStr">
+      <c r="C29" s="36" t="inlineStr">
         <is>
           <t>$2312.5M to be recognized over 24-36 months of construction</t>
         </is>
@@ -6962,7 +7050,7 @@
           <t>Escrow Bank Protection</t>
         </is>
       </c>
-      <c r="C30" s="35" t="inlineStr">
+      <c r="C30" s="36" t="inlineStr">
         <is>
           <t>100.0% of buyer presale funds deposited in RERA statutory escrow bank accounts</t>
         </is>
@@ -6974,7 +7062,7 @@
           <t>Milestone Collection Cycle</t>
         </is>
       </c>
-      <c r="C31" s="35" t="inlineStr">
+      <c r="C31" s="36" t="inlineStr">
         <is>
           <t>Construction-linked milestone payment structures (Average 30% downpayment / 70% handover)</t>
         </is>
@@ -7006,7 +7094,7 @@
           <t>Unrestricted Treasury Cash</t>
         </is>
       </c>
-      <c r="C35" s="35" t="inlineStr">
+      <c r="C35" s="36" t="inlineStr">
         <is>
           <t>$185.2M in central treasury accounts</t>
         </is>
@@ -7018,7 +7106,7 @@
           <t>Restricted Escrow Bank Balances</t>
         </is>
       </c>
-      <c r="C36" s="35" t="inlineStr">
+      <c r="C36" s="36" t="inlineStr">
         <is>
           <t>$242.2M ring-fenced for specific project construction works</t>
         </is>
@@ -7030,7 +7118,7 @@
           <t>Undrawn Committed Bank Rcfs</t>
         </is>
       </c>
-      <c r="C37" s="35" t="inlineStr">
+      <c r="C37" s="36" t="inlineStr">
         <is>
           <t>$218.1M in bilateral bank revolving credit lines</t>
         </is>
@@ -7042,18 +7130,142 @@
           <t>Total Available Liquidity Runway</t>
         </is>
       </c>
-      <c r="C38" s="35" t="inlineStr">
+      <c r="C38" s="36" t="inlineStr">
         <is>
           <t>42 months of corporate debt service and fixed overhead pre-funded</t>
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>VI. BRANDED LUXURY RESIDENCES PORTFOLIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Operational Asset / Disclosure Dimension</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Conference Call &amp; Investor Deck Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Bugatti Residences By Binghatti</t>
+        </is>
+      </c>
+      <c r="C41" s="36" t="inlineStr">
+        <is>
+          <t>Ultra-luxury 46-story tower in Business Bay with 182 bespoke units; penthouse sales exceeding AED 9,500/sqft; 100% sold out in phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Mercedes Benz Places</t>
+        </is>
+      </c>
+      <c r="C42" s="36" t="inlineStr">
+        <is>
+          <t>65-story residential icon in Downtown Dubai overlooking Burj Khalifa; total GDV of AED 3.6B ($980M); presales velocity &gt;85% in first 90 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Burj Binghatti Jacob And Co</t>
+        </is>
+      </c>
+      <c r="C43" s="36" t="inlineStr">
+        <is>
+          <t>Ultra-tall branded residential hyper-tower competing for world's tallest residential crown; exclusive high-net-worth buyer demand from GCC, Europe, and Asia</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Branded Sales Margin Premium</t>
+        </is>
+      </c>
+      <c r="C44" s="36" t="inlineStr">
+        <is>
+          <t>Branded residences achieve 42% - 48% gross margins vs 28% - 32% on standard signature off-plan developments</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>VII. RERA ESCROW AND INVESTOR PROTECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Operational Asset / Disclosure Dimension</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Conference Call &amp; Investor Deck Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Escrow Bank Protection</t>
+        </is>
+      </c>
+      <c r="C48" s="36" t="inlineStr">
+        <is>
+          <t>100% of buyer off-plan payments are deposited directly into designated RERA-monitored escrow accounts at top-tier UAE banks (Emirates NBD, FAB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Escrow Disbursement Gating</t>
+        </is>
+      </c>
+      <c r="C49" s="36" t="inlineStr">
+        <is>
+          <t>Funds can only be withdrawn upon audited civil engineering milestone completion verified by Dubai Land Department engineers</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Sukuk Payback Liquidity</t>
+        </is>
+      </c>
+      <c r="C50" s="36" t="inlineStr">
+        <is>
+          <t>Existing cash balance ($245M) + audited escrow receivables ($490M) cover 2.6x the total 2027 Sukuk principal ($280M)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="35">
     <mergeCell ref="C36:I36"/>
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="C17:I17"/>
+    <mergeCell ref="C48:I48"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="C38:I38"/>
     <mergeCell ref="C19:I19"/>
@@ -7061,21 +7273,29 @@
     <mergeCell ref="C28:I28"/>
     <mergeCell ref="C18:I18"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C49:I49"/>
     <mergeCell ref="F11:I11"/>
     <mergeCell ref="C34:I34"/>
     <mergeCell ref="C24:I24"/>
     <mergeCell ref="C30:I30"/>
+    <mergeCell ref="C42:I42"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="C14:I14"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="C35:I35"/>
     <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C47:I47"/>
     <mergeCell ref="C16:I16"/>
     <mergeCell ref="C25:I25"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C50:I50"/>
     <mergeCell ref="C31:I31"/>
+    <mergeCell ref="C44:I44"/>
     <mergeCell ref="C22:I22"/>
+    <mergeCell ref="C40:I40"/>
     <mergeCell ref="F8:I8"/>
+    <mergeCell ref="C43:I43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>